<commit_message>
Publish bilingual bank evidence package
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-fi.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-fi.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=event ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=doclist ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf</t>
+          <t>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=event ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=doclist ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB1/document.pdf ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Saksan mitätöintikanne hylättiin 14.1.2026, mutta valitus on vireillä.</t>
+          <t>Saksan virallinen tapahtuma: Mitätöintikanne hylättiin; valitus vireillä (14.1.2026).</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Väite rajataan Saksan osaan ja nykyiseen prosessitilaan.</t>
+          <t>Maantieteellinen ja prosessuaalinen rajaus: Saksa. Ei lainvoimainen BGH-valituksen ollessa vireillä.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -897,14 +897,14 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Seuraa BGH-valituksen X ZR 21/26 etenemistä ja lopputulosta.</t>
+          <t>Seuraa muutoksenhakua X ZR 21/26, sen lopputulosta, täytäntöönpanoa ja mahdollisia maksettuja korvauksia.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Münchenin tuomioistuin totesi tarkasteltujen tuotteiden loukkaavan vaatimuksia 1 ja 6.</t>
+          <t>Saksan virallinen tapahtuma koski vaatimuksia 1 ja 6: Tarkasteltujen tuotteiden todettiin loukkaavan patenttia.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Ei yleistetä muihin tuotteisiin, yhtiöihin tai maihin.</t>
+          <t>Maantieteellinen ja prosessuaalinen rajaus: Saksa. Virallinen tuomio on saatavilla; valitustilaa, lainvoimaisuutta ja täytäntöönpanoa ei ole tässä julkaisussa riippumattomasti vahvistettu.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -944,14 +944,14 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Valitustila, lainvoimaisuus, täytäntöönpano ja maksetut korvaukset on vahvistettava.</t>
+          <t>Vahvista valitustila, lainvoimaisuus, täytäntöönpano ja maksetut korvaukset.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kiinan tunnistettu asia on hakijapuolen uudelleentarkastus, ei loukkausoikeudenkäynti.</t>
+          <t>Kiinan tunnistettu menettely: Kiinan hakijapuolen uudelleentarkastus tunnistettu; perusteluja ei saatu.</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365 ; https://www.cnipa.gov.cn/art/2020/6/5/art_1517_92474.html</t>
+          <t>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365 ; https://www.cnipa.gov.cn/art/2020/6/5/art_1517_92474.html ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Kolme yksittäistä verkkokauppahintaa; vuosiero; vain verotettu neste.</t>
+          <t>Kolme yksittäistä verkkokauppahintaa; syötevuodet 2025 ja 2026; vain verotettu neste.</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Tarvitaan edustava hintakori, tuotemix, kanavamarginaalit ja saman vuoden hinnat.</t>
+          <t>Tarvitaan edustava hintakori, tuotemix ja kanavamarginaalit sekä mallivuoden 2025 hinnat.</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Neljä rekisteritarkistusta ei kata koko perhettä.</t>
+          <t>Neljä kansallista rekisterijurisdiktiota ei kata koko perhettä.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851</t>
+          <t>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>2026.07.22-7</t>
+          <t>2026.07.22-8</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish bilingual bank evidence package (#6)
Release bilingual 6/12/30-slide diligence decks, Evidence Registers, draft-only official-data request programme, browser integrity verification and privacy hardening.
</commit_message>
<xml_diff>
--- a/site/downloads/pixan-bank-evidence-register-fi.xlsx
+++ b/site/downloads/pixan-bank-evidence-register-fi.xlsx
@@ -731,7 +731,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=event ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=doclist ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf</t>
+          <t>https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=event ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=doclist ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB1/document.pdf ; https://data.epo.org/publication-server/rest/v1.2/patents/EP3032975NWB2/document.pdf</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -857,7 +857,7 @@
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Saksan mitätöintikanne hylättiin 14.1.2026, mutta valitus on vireillä.</t>
+          <t>Saksan virallinen tapahtuma: Mitätöintikanne hylättiin; valitus vireillä (14.1.2026).</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Väite rajataan Saksan osaan ja nykyiseen prosessitilaan.</t>
+          <t>Maantieteellinen ja prosessuaalinen rajaus: Saksa. Ei lainvoimainen BGH-valituksen ollessa vireillä.</t>
         </is>
       </c>
       <c r="H7" s="3" t="inlineStr">
@@ -897,14 +897,14 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Seuraa BGH-valituksen X ZR 21/26 etenemistä ja lopputulosta.</t>
+          <t>Seuraa muutoksenhakua X ZR 21/26, sen lopputulosta, täytäntöönpanoa ja mahdollisia maksettuja korvauksia.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Münchenin tuomioistuin totesi tarkasteltujen tuotteiden loukkaavan vaatimuksia 1 ja 6.</t>
+          <t>Saksan virallinen tapahtuma koski vaatimuksia 1 ja 6: Tarkasteltujen tuotteiden todettiin loukkaavan patenttia.</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -934,7 +934,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Ei yleistetä muihin tuotteisiin, yhtiöihin tai maihin.</t>
+          <t>Maantieteellinen ja prosessuaalinen rajaus: Saksa. Virallinen tuomio on saatavilla; valitustilaa, lainvoimaisuutta ja täytäntöönpanoa ei ole tässä julkaisussa riippumattomasti vahvistettu.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
@@ -944,14 +944,14 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Valitustila, lainvoimaisuus, täytäntöönpano ja maksetut korvaukset on vahvistettava.</t>
+          <t>Vahvista valitustila, lainvoimaisuus, täytäntöönpano ja maksetut korvaukset.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Kiinan tunnistettu asia on hakijapuolen uudelleentarkastus, ei loukkausoikeudenkäynti.</t>
+          <t>Kiinan tunnistettu menettely: Kiinan hakijapuolen uudelleentarkastus tunnistettu; perusteluja ei saatu.</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -966,7 +966,7 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365 ; https://www.cnipa.gov.cn/art/2020/6/5/art_1517_92474.html</t>
+          <t>https://litigation.rpxcorp.com/china/prb/5153434-picsen-company-v-pixan-oy-of-365 ; https://www.cnipa.gov.cn/art/2020/6/5/art_1517_92474.html ; https://register.epo.org/application?number=EP14836345&amp;lng=en&amp;tab=family</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Kolme yksittäistä verkkokauppahintaa; vuosiero; vain verotettu neste.</t>
+          <t>Kolme yksittäistä verkkokauppahintaa; syötevuodet 2025 ja 2026; vain verotettu neste.</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>Tarvitaan edustava hintakori, tuotemix, kanavamarginaalit ja saman vuoden hinnat.</t>
+          <t>Tarvitaan edustava hintakori, tuotemix ja kanavamarginaalit sekä mallivuoden 2025 hinnat.</t>
         </is>
       </c>
     </row>
@@ -1921,7 +1921,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Neljä rekisteritarkistusta ei kata koko perhettä.</t>
+          <t>Neljä kansallista rekisterijurisdiktiota ei kata koko perhettä.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
@@ -2282,7 +2282,7 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851</t>
+          <t>https://fees.uspto.gov/MaintenanceFees/fees/details?patentNumber=10306923 ; https://patentcenter.uspto.gov/applications/14911851 ; https://assignment.uspto.gov/patent/index.html#/patent/search/resultFilter?searchInput=10306923</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
@@ -2779,7 +2779,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>2026.07.22-7</t>
+          <t>2026.07.22-8</t>
         </is>
       </c>
     </row>

</xml_diff>